<commit_message>
Cores da marca Nossa Saude e nomes de arquivo amigaveis
Site e PDFs passam a usar a paleta oficial da operadora (nossasaude.com.br):
petroleo #004159 / #006285 e laranja #F07F09 / #E6411C, com neutros mornos
derivados do #4C4441 do texto deles. O selo dourado continua sendo a
assinatura da Mazza Broker.

Os guias agora salvam como "Nossa Saude - <Cidade>.pdf" (atributo download nos
links; a URL segue sem acento) e os arquivos do estudo foram renomeados no
mesmo padrao.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/arquivos/rede-nossa-saude-campos-gerais.xlsx
+++ b/arquivos/rede-nossa-saude-campos-gerais.xlsx
@@ -48,16 +48,16 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="FF0D2A4F"/>
+      <color rgb="FF004159"/>
       <sz val="18"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="FF9A7513"/>
+      <color rgb="FFF07F09"/>
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="FF89909C"/>
+      <color rgb="FF8B8580"/>
       <sz val="10"/>
     </font>
     <font>
@@ -74,12 +74,12 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="FF0D2A4F"/>
+      <color rgb="FF004159"/>
       <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="FF0D2A4F"/>
+      <color rgb="FF004159"/>
       <sz val="16"/>
     </font>
     <font>
@@ -89,7 +89,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="FF9A7513"/>
+      <color rgb="FFF07F09"/>
       <sz val="10"/>
     </font>
     <font>
@@ -117,17 +117,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0D2A4F"/>
+        <fgColor rgb="FF004159"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF9A7513"/>
+        <fgColor rgb="FFF07F09"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF7F8FB"/>
+        <fgColor rgb="FFF5F8F9"/>
       </patternFill>
     </fill>
   </fills>
@@ -141,16 +141,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFE2E6EC"/>
+        <color rgb="FFE3E0DC"/>
       </left>
       <right style="thin">
-        <color rgb="FFE2E6EC"/>
+        <color rgb="FFE3E0DC"/>
       </right>
       <top style="thin">
-        <color rgb="FFE2E6EC"/>
+        <color rgb="FFE3E0DC"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFE2E6EC"/>
+        <color rgb="FFE3E0DC"/>
       </bottom>
     </border>
   </borders>

</xml_diff>